<commit_message>
tableau: portable metric contract, generated four-dashboard workbook, docs and pipeline steps
- metrics/semantic_layer.yml: semantic models, entities, dimensions, measures and governed metrics with the full KPI
  contract; src/validation/semantic_layer.py ties every metric-month to the marts and generates the metric dictionary
- fix: mart_revenue_kpis average per active row divided by one row per month; now uses active customers
- src/tableau: governed extracts, four dashboards with Hyper extracts, manifest, expected KPIs and a tie-out
- tests for duplicate metrics, bridge roll-forward, retention bounds, invoice arithmetic, zero denominators,
  KPI drift, manifest integrity and disclaimers; make pipeline runs the contract and Tableau steps
- README title: MRR, Retention & Billing Controls; Tableau status stated as not yet published
</commit_message>
<xml_diff>
--- a/excel/finance_reconciliation.xlsx
+++ b/excel/finance_reconciliation.xlsx
@@ -679,7 +679,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-09-19 20:00</t>
+          <t>2026-09-19 20:07</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>69af662c7932</t>
+          <t>a13e601c1309</t>
         </is>
       </c>
     </row>
@@ -895,7 +895,7 @@
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;9 SaaS Revenue Intelligence | MRR, Retention &amp;&amp; Billing Controls&amp;R&amp;9 Control</oddHeader>
-    <oddFooter>&amp;L&amp;8 Synthetic data. Not real financial results.&amp;C&amp;8 Refreshed 2026-09-19 20:00 UTC&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 Synthetic data. Not real financial results.&amp;C&amp;8 Refreshed 2026-09-19 20:07 UTC&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3125,7 +3125,7 @@
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;9 SaaS Revenue Intelligence | MRR, Retention &amp;&amp; Billing Controls&amp;R&amp;9 MRR Bridge</oddHeader>
-    <oddFooter>&amp;L&amp;8 Synthetic data. Not real financial results.&amp;C&amp;8 Refreshed 2026-09-19 20:00 UTC&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 Synthetic data. Not real financial results.&amp;C&amp;8 Refreshed 2026-09-19 20:07 UTC&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -5073,7 +5073,7 @@
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;9 SaaS Revenue Intelligence | MRR, Retention &amp;&amp; Billing Controls&amp;R&amp;9 Billing Reconciliation</oddHeader>
-    <oddFooter>&amp;L&amp;8 Synthetic data. Not real financial results.&amp;C&amp;8 Refreshed 2026-09-19 20:00 UTC&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 Synthetic data. Not real financial results.&amp;C&amp;8 Refreshed 2026-09-19 20:07 UTC&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -37194,7 +37194,7 @@
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;9 SaaS Revenue Intelligence | MRR, Retention &amp;&amp; Billing Controls&amp;R&amp;9 Exceptions</oddHeader>
-    <oddFooter>&amp;L&amp;8 Synthetic data. Not real financial results.&amp;C&amp;8 Refreshed 2026-09-19 20:00 UTC&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 Synthetic data. Not real financial results.&amp;C&amp;8 Refreshed 2026-09-19 20:07 UTC&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -37318,7 +37318,7 @@
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;9 SaaS Revenue Intelligence | MRR, Retention &amp;&amp; Billing Controls&amp;R&amp;9 Scenario Inputs</oddHeader>
-    <oddFooter>&amp;L&amp;8 Synthetic data. Not real financial results.&amp;C&amp;8 Refreshed 2026-09-19 20:00 UTC&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 Synthetic data. Not real financial results.&amp;C&amp;8 Refreshed 2026-09-19 20:07 UTC&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -38935,7 +38935,7 @@
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;9 SaaS Revenue Intelligence | MRR, Retention &amp;&amp; Billing Controls&amp;R&amp;9 Scenario Output</oddHeader>
-    <oddFooter>&amp;L&amp;8 Synthetic data. Not real financial results.&amp;C&amp;8 Refreshed 2026-09-19 20:00 UTC&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 Synthetic data. Not real financial results.&amp;C&amp;8 Refreshed 2026-09-19 20:07 UTC&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -39173,7 +39173,7 @@
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;9 SaaS Revenue Intelligence | MRR, Retention &amp;&amp; Billing Controls&amp;R&amp;9 Metric Definitions</oddHeader>
-    <oddFooter>&amp;L&amp;8 Synthetic data. Not real financial results.&amp;C&amp;8 Refreshed 2026-09-19 20:00 UTC&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 Synthetic data. Not real financial results.&amp;C&amp;8 Refreshed 2026-09-19 20:07 UTC&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>